<commit_message>
Actualizacao do layout das poupancas
</commit_message>
<xml_diff>
--- a/Grupos_Poupanca.xlsx
+++ b/Grupos_Poupanca.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -399,334 +399,670 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OFENSIVA</t>
+          <t>NACARROANE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>3918786000010250018</t>
+          <t>3918786000010254048</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Aurélio António</t>
+          <t>Manuel Caetano</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>FUTURO MELHOR</t>
+          <t>Somos Caz 2</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>OFENSIVA</t>
+          <t>NACARROANE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3918786000010250016</t>
+          <t>3918786000010254046</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Aurélio António</t>
+          <t>Manuel Caetano</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>MAIS FORCA</t>
+          <t>Somos Capaz</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>OFENSIVA</t>
+          <t>NAMARIESSA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3918786000010250014</t>
+          <t>3918786000010254044</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Aurélio António</t>
+          <t>Manuel Caetano</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>Poupança da Sorte</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NICANE</t>
+          <t>CURRAPE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3918786000010250012</t>
+          <t>3918786000010254042</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Aurélio António</t>
+          <t>Manuel Caetano</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>UNIAO FAZ A FORCA</t>
+          <t>Ossuka</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NICANE</t>
+          <t>CURRAPE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3918786000010250010</t>
+          <t>3918786000010254040</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Aurélio António</t>
+          <t>Manuel Caetano</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>ORUWERA</t>
+          <t>Inthela</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NICANE</t>
+          <t>MICUE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3918786000010250008</t>
+          <t>3918786000010254038</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Aurélio António</t>
+          <t>Manuel Caetano</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>MUDANCA DE VIDA</t>
+          <t>Ochutha Ossuka</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>39</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MURROMONE</t>
+          <t>NAMUALI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3918786000010250006</t>
+          <t>3918786000010254036</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Ribaue</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Aurélio António</t>
+          <t>Manuel Caetano</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>MUATHUNAKA</t>
+          <t>Wiwanana</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>25</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NAMALE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>3918786000010254034</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ribaue</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Manuel Caetano</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">União Faz A força </t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>OFENSIVA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>3918786000010250018</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>FUTURO MELHOR</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>OFENSIVA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>3918786000010250016</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>MAIS FORCA</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>OFENSIVA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>3918786000010250014</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>UNIDADE</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NICANE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>3918786000010250012</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>UNIAO FAZ A FORCA</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>NICANE</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>3918786000010250010</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>ORUWERA</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NICANE</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>3918786000010250008</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>MUDANCA DE VIDA</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MURROMONE</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>3918786000010250006</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Aurélio António</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>MUATHUNAKA</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>25</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>JARDIM</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>3918786000010250004</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Monapo</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Aurélio António</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>WIKHALIHERA</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>27</t>
         </is>
@@ -735,271 +1071,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="481cb719fb2f51215cc00c8d40533043">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="71df0815368817fe9627576b1e062219" ns2:_="" ns3:_="">
-    <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
-    <xsd:import namespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="20d57abc-823c-4051-a81a-1a0a01a8f39e" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="16" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="22" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{21a739d7-e82a-41d6-a891-a689fdcdcba6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="54c5ab46-7543-4aba-b0fa-79d6a199bef5">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{428A1417-8FE6-4BD6-B688-9FC66B5F33DA}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11B9D858-BF36-44EC-9C39-BCD247F2B2A6}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{61470D7A-0FED-40B4-9468-120F986E1DE4}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao grafico de poupanças
</commit_message>
<xml_diff>
--- a/Grupos_Poupanca.xlsx
+++ b/Grupos_Poupanca.xlsx
@@ -1329,13 +1329,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{134B2349-C2E8-4EC3-A04E-73FB3C6D0F45}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{778A27BE-88E7-44F8-8998-FE41F58F408E}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2DBACE48-429E-4A87-A282-7F82AC3BDBA5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69CAE2BA-21CC-4768-9E5E-3C7EBECF3A14}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{25A21929-82B3-4393-9CA9-5C88ED9AB4DB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FB78DE61-A1DC-41A1-996C-4C43225BB85D}"/>
 </file>
</xml_diff>